<commit_message>
Update tracker and create v5 plan with revised architecture
- Tracker: Mark 0.8, 0.9, 0.10, 0.6 as Done. Revise Phase 1 tasks.
- Plan v5: Pipedrive as single source of truth for contact data.
  Leads table stores intelligence only. Campaign config replaces
  contact pool. Auto-fill call queue from Pipedrive filters.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Operational_Readiness_Tracker.xlsx
+++ b/docs/Operational_Readiness_Tracker.xlsx
@@ -853,10 +853,14 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Was already implemented correctly in code</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -901,10 +905,14 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Backend code done, frontend compatibility fix applied. Build/bundle issue under investigation.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -949,12 +957,12 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Run drizzle-kit push after</t>
+          <t>Schema pushed, columns verified in DB</t>
         </is>
       </c>
     </row>
@@ -1001,10 +1009,14 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Schema pushed, seed data migrated via SQL script</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1049,10 +1061,14 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Schema pushed, table verified in DB</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add v6 plan: app owns data, Aircall dispatch, Pipedrive push for qualified only
Architecture reversal: app is single source of truth for all contacts.
CSV upload to local pool, dispatch to Aircall power dialer, only
interested/meeting-booked outcomes push to Pipedrive. Two-table model:
contacts (full pool) + leads (intelligence layer).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Operational_Readiness_Tracker.xlsx
+++ b/docs/Operational_Readiness_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Implementation Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="New Files" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Modified Files" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Environment Variables" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Phase Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New Files" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modified Files" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment Variables" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Implementation Tracker'!$A$1:$J$1</definedName>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1367,54 +1367,52 @@
       <c r="J17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>2.1</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Aircall: design constraints (research)</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Document Aircall API behavior: no transcript in call.ended, tags arrive late, transcription needs AI Assist.</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>Must understand API before building. Wrong assumptions = broken integration.</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>N/A (documented in plan)</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="A18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Pipedrive push service</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>One-way push on interested/meeting-booked. Create person + deal in Pipedrive. Store IDs on contact record. No sync, no cache.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Only qualified leads enter Pipedrive. Keeps it clean.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>lib/pipedrivePushService.ts, routes/pipedrive/index.ts</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Research complete</t>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>v6: NEW. Simple one-way push.</t>
         </is>
       </c>
     </row>
@@ -1426,37 +1424,37 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Aircall: transcription service</t>
+          <t>Aircall: design constraints (research)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Two paths: AI Assist (webhook) or external (download MP3 + Whisper/Deepgram). Config-driven.</t>
+          <t>Document Aircall API behavior: no transcript in call.ended, tags arrive late, transcription needs AI Assist.</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>call.ended has no transcript. Must handle transcription separately.</t>
+          <t>Must understand API before building. Wrong assumptions = broken integration.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Config</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>lib/transcriptionService.ts</t>
+          <t>N/A (documented in plan)</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>None</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1466,7 +1464,7 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Env: AIRCALL_TRANSCRIPTION_MODE, TRANSCRIPTION_API_KEY</t>
+          <t>Research complete</t>
         </is>
       </c>
     </row>
@@ -1478,37 +1476,37 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Aircall: extract transcript utils</t>
+          <t>Aircall: transcription service</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Move isAircallFormat, normaliseAircallTranscript, identifyAgentLabel to shared utility.</t>
+          <t>Two paths: AI Assist (webhook) or external (download MP3 + Whisper/Deepgram). Config-driven.</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>These functions are embedded in recommendation route. Need them in webhook handler too.</t>
+          <t>call.ended has no transcript. Must handle transcription separately.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Utility</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>lib/aircallTranscriptUtils.ts, routes/recommendation/index.ts</t>
+          <t>lib/transcriptionService.ts</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -1516,7 +1514,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Env: AIRCALL_TRANSCRIPTION_MODE, TRANSCRIPTION_API_KEY</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1526,37 +1528,37 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Aircall: call outcome service</t>
+          <t>Aircall: extract transcript utils</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Map tags to actions. TAG_MAPPING config object. interested/no-interest/meeting-booked/no-answer/callback/not-now.</t>
+          <t>Move isAircallFormat, normaliseAircallTranscript, identifyAgentLabel to shared utility.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Without outcomes, leads stay in same state regardless of call result. Loop doesn't close.</t>
+          <t>These functions are embedded in recommendation route. Need them in webhook handler too.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>lib/callOutcomeService.ts</t>
+          <t>lib/aircallTranscriptUtils.ts, routes/recommendation/index.ts</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>0.8, 0.10</t>
+          <t>None</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1564,11 +1566,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>Case-insensitive tag mapping</t>
-        </is>
-      </c>
+      <c r="J21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1578,37 +1576,37 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Aircall: webhook handler</t>
+          <t>Aircall: call outcome service</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>POST /aircall/webhook handling call.ended, call.tagged, transcription.created events.</t>
+          <t>Map tags to actions. TAG_MAPPING config object. interested/no-interest/meeting-booked/no-answer/callback/not-now.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Need to receive Aircall events automatically instead of manual file upload.</t>
+          <t>Without outcomes, leads stay in same state regardless of call result. Loop doesn't close.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>routes/aircall/index.ts, routes/index.ts</t>
+          <t>lib/callOutcomeService.ts</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2.2, 2.3, 2.4</t>
+          <t>0.8, 0.10</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -1618,7 +1616,7 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Env: AIRCALL_WEBHOOK_TOKEN, AIRCALL_API_ID, AIRCALL_API_TOKEN</t>
+          <t>v6: interested/meeting-booked also trigger Pipedrive push (1.6)</t>
         </is>
       </c>
     </row>
@@ -1630,22 +1628,22 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Fireflies: webhook handler</t>
+          <t>Aircall: webhook handler</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>POST /fireflies/webhook. Match by participant email. Create lead_conversations, trigger pipeline.</t>
+          <t>POST /aircall/webhook handling call.ended, call.tagged, transcription.created events.</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Google Meet transcripts must flow automatically. Manual paste = inconsistent logging.</t>
+          <t>Need to receive Aircall events automatically instead of manual file upload.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1655,12 +1653,12 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>routes/fireflies/index.ts, routes/index.ts</t>
+          <t>routes/aircall/index.ts, routes/index.ts</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>0.10, 0.5</t>
+          <t>2.2, 2.3, 2.4</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -1670,7 +1668,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Env: FIREFLIES_WEBHOOK_SECRET</t>
+          <t>v6: Outcomes reference local contacts table</t>
         </is>
       </c>
     </row>
@@ -1682,37 +1680,37 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>2.7a</t>
+          <t>2.6</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Google Calendar: API client</t>
+          <t>Fireflies: webhook handler</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Create lib/integrations/google-calendar/ with OAuth flow, event CRUD, date range queries.</t>
+          <t>POST /fireflies/webhook. Match by participant email. Create lead_conversations, trigger pipeline.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Need Calendar API access for meeting and callback invites.</t>
+          <t>Google Meet transcripts must flow automatically. Manual paste = inconsistent logging.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>lib/integrations/google-calendar/src/client.ts</t>
+          <t>routes/fireflies/index.ts, routes/index.ts</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>0.10, 0.5</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -1722,7 +1720,7 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Env: GOOGLE_CALENDAR_CLIENT_ID/SECRET/REDIRECT</t>
+          <t>Env: FIREFLIES_WEBHOOK_SECRET</t>
         </is>
       </c>
     </row>
@@ -1734,37 +1732,37 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>2.7b</t>
+          <t>2.7a</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Google Calendar: calendar service</t>
+          <t>Google Calendar: API client</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>createMeetingEvent, createCallbackEvent, createFollowUpEvent, getEventsForDate.</t>
+          <t>Create lib/integrations/google-calendar/ with OAuth flow, event CRUD, date range queries.</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Outcome dialog needs to auto-create calendar events for meetings and callbacks.</t>
+          <t>Need Calendar API access for meeting and callback invites.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>lib/calendarService.ts</t>
+          <t>lib/integrations/google-calendar/src/client.ts</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2.7a</t>
+          <t>None</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -1772,7 +1770,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Env: GOOGLE_CALENDAR_CLIENT_ID/SECRET/REDIRECT</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1782,37 +1784,37 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>2.7c</t>
+          <t>2.7b</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Google Calendar: outcome dialog</t>
+          <t>Google Calendar: calendar service</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Add date/time picker to outcome dialog. Auto-create calendar event for meeting-booked and callback-requested.</t>
+          <t>createMeetingEvent, createCallbackEvent, createFollowUpEvent, getEventsForDate.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Investors need calendar invites. No invite = nothing in their diary.</t>
+          <t>Outcome dialog needs to auto-create calendar events for meetings and callbacks.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>pages/call-prep.tsx, pages/call-inbox.tsx</t>
+          <t>lib/calendarService.ts</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>2.7b, 2.4</t>
+          <t>2.7a</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -1830,22 +1832,22 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>2.8a</t>
+          <t>2.7c</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Frontend: Call Inbox page</t>
+          <t>Google Calendar: outcome dialog</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>New page listing all conversations. Source icons, status indicators, filters, manual link, reprocess.</t>
+          <t>Add date/time picker to outcome dialog. Auto-create calendar event for meeting-booked and callback-requested.</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Need visibility of all calls/meetings across sources with status tracking.</t>
+          <t>Investors need calendar invites. No invite = nothing in their diary.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1855,12 +1857,12 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>pages/call-inbox.tsx, components/layout.tsx, App.tsx</t>
+          <t>pages/call-prep.tsx, pages/call-inbox.tsx</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>2.5, 2.6</t>
+          <t>2.7b, 2.4</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -1878,93 +1880,93 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
+          <t>2.8a</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Frontend: Call Inbox page</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>New page listing all conversations. Source icons, status indicators, filters, manual link, reprocess.</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Need visibility of all calls/meetings across sources with status tracking.</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>pages/call-inbox.tsx, components/layout.tsx, App.tsx</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>2.5, 2.6</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
           <t>2.8b</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Frontend: Lead detail updates</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Add Log Meeting button, Conversations section with summaries, belief diffs, intelligence delta.</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>Lead detail needs conversation history and what-changed views.</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>pages/lead-detail.tsx</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>0.10, 0.11</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Pipeline: job tracking schema</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>pipeline_jobs table with batch_id, job_type, status, lead_id, attempts, timestamps.</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Need persistent job tracking for batch processing.</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Schema</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>lib/db/src/schema/pipeline-jobs.ts</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1974,37 +1976,37 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Pipeline: queue service + orphan recovery</t>
+          <t>Pipeline: job tracking schema</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>pipelineQueue.ts using batchProcess utility. Startup recovery, 60s polling, heartbeat.</t>
+          <t>pipeline_jobs table with batch_id, job_type, status, lead_id, attempts, timestamps.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Replit may kill processes mid-batch. Must detect and recover orphaned jobs.</t>
+          <t>Need persistent job tracking for batch processing.</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Schema</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>lib/pipelineQueue.ts</t>
+          <t>lib/db/src/schema/pipeline-jobs.ts</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>3.1, 0.2</t>
+          <t>None</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
@@ -2022,97 +2024,93 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Pipeline: queue service + orphan recovery</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>pipelineQueue.ts using batchProcess utility. Startup recovery, 60s polling, heartbeat.</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Replit may kill processes mid-batch. Must detect and recover orphaned jobs.</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>lib/pipelineQueue.ts</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>3.1, 0.2</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Pipeline: API routes + frontend</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>POST /enqueue, GET /status, GET /jobs. Bulk Run Pipeline actions on leads + contact pool. Progress banner.</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>Need to enqueue hundreds of leads and track progress.</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>Route + Frontend</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>routes/pipeline/index.ts, pages/leads.tsx, pages/contact-pool.tsx</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>3.2, 0.7</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
+      <c r="I32" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J31" s="5" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>4.1</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>Belief-driven call prep page</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Complete redesign: qualification gates, belief map with questions, context (summaries, sent docs, objections), action buttons.</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Caller needs belief map as primary interface before every call. Current page is generic 4 questions.</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>pages/call-prep.tsx, routes/leads/index.ts (call-prep endpoint)</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>0.9, 0.10, 0.11</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t>THE primary interface</t>
-        </is>
-      </c>
+      <c r="J32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -2122,37 +2120,37 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Daily call queue page</t>
+          <t>Belief-driven call prep page</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>New page: prioritised list (callbacks, interested, cold at sequence day, re-entries). Re-entry reset at query time.</t>
+          <t>Complete redesign: qualification gates, belief map with questions, context (summaries, sent docs, objections), action buttons.</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Caller needs to know who to call each morning. Currently no prioritised list.</t>
+          <t>Caller needs belief map as primary interface before every call. Current page is generic 4 questions.</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Frontend + Route</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>pages/call-queue.tsx, routes/leads/index.ts (call-queue endpoint)</t>
+          <t>pages/call-prep.tsx, routes/leads/index.ts (call-prep endpoint)</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>2.4, 0.8</t>
+          <t>0.9, 0.10, 0.11</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2162,7 +2160,7 @@
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>Re-entry flips paused-&gt;active at query time</t>
+          <t>THE primary interface</t>
         </is>
       </c>
     </row>
@@ -2174,22 +2172,22 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Dashboard: campaign wave tracking</t>
+          <t>Daily call queue page</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Widget showing active wave, dispatched today/week, total in wave, remaining in pool.</t>
+          <t>New page: prioritised list (callbacks, interested, cold at sequence day, re-entries). Re-entry reset at query time.</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Team needs to see where they are in the 25K campaign.</t>
+          <t>Caller needs to know who to call each morning. Currently no prioritised list.</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -2199,12 +2197,12 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>pages/dashboard.tsx, routes/dashboard/index.ts</t>
+          <t>pages/call-queue.tsx, routes/leads/index.ts (call-queue endpoint)</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>2.4, 0.8</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
@@ -2212,7 +2210,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J34" s="6" t="inlineStr"/>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>Re-entry flips paused-&gt;active at query time</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -2222,22 +2224,22 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Dashboard: funnel view</t>
+          <t>Dashboard: campaign wave tracking</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Counts by pipeline_stage. Plus terminal states (Closed, Paused, Passive).</t>
+          <t>Widget showing active wave, dispatched today/week, total in wave, remaining in pool.</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Need 'where is everyone right now' at a glance.</t>
+          <t>Team needs to see where they are in the 25K campaign.</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -2270,22 +2272,22 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Dashboard: error visibility</t>
+          <t>Dashboard: funnel view</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>'X items need attention' widget. Failed jobs, syncs, unmatched calls, unprocessed outcomes.</t>
+          <t>Counts by pipeline_stage. Plus terminal states (Closed, Paused, Passive).</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Silent failures where leads fall through cracks is worst outcome.</t>
+          <t>Need 'where is everyone right now' at a glance.</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2300,7 +2302,7 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>2.5, 3.1</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2318,37 +2320,37 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Enhanced lead detail timeline</t>
+          <t>Dashboard: error visibility</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Unified timeline: stage changes, conversations, sends, belief transitions, intelligence updates.</t>
+          <t>'X items need attention' widget. Failed jobs, syncs, unmatched calls, unprocessed outcomes.</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Need complete chronological interaction history per lead.</t>
+          <t>Silent failures where leads fall through cracks is worst outcome.</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Frontend + Route</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>pages/lead-detail.tsx</t>
+          <t>pages/dashboard.tsx, routes/dashboard/index.ts</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>0.10, 2.4</t>
+          <t>2.5, 3.1</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
@@ -2366,37 +2368,37 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Content routing audit</t>
+          <t>Enhanced lead detail timeline</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Review recommendation route. Ensure belief gates are primary driver, stage is sanity check only.</t>
+          <t>Unified timeline: stage changes, conversations, sends, belief transitions, intelligence updates.</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Stage currently filters content alongside beliefs. Beliefs should be primary.</t>
+          <t>Need complete chronological interaction history per lead.</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Review + Fix</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>routes/recommendation/index.ts</t>
+          <t>pages/lead-detail.tsx</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>0.10, 2.4</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2404,11 +2406,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J38" s="6" t="inlineStr">
-        <is>
-          <t>Review task, not rewrite</t>
-        </is>
-      </c>
+      <c r="J38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -2418,37 +2416,37 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Belief system admin page</t>
+          <t>Content routing audit</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>New page: belief registry editor, document-to-belief matrix, gate rules overview.</t>
+          <t>Review recommendation route. Ensure belief gates are primary driver, stage is sanity check only.</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Non-developers can't adjust beliefs, questions, gates, or content mappings without code.</t>
+          <t>Stage currently filters content alongside beliefs. Beliefs should be primary.</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Review + Fix</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>pages/belief-admin.tsx, components/layout.tsx, App.tsx</t>
+          <t>routes/recommendation/index.ts</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>None</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -2456,7 +2454,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J39" s="6" t="inlineStr"/>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>Review task, not rewrite</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -2466,99 +2468,95 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Belief system admin page</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>New page: belief registry editor, document-to-belief matrix, gate rules overview.</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Non-developers can't adjust beliefs, questions, gates, or content mappings without code.</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>pages/belief-admin.tsx, components/layout.tsx, App.tsx</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
           <t>4.9</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>Content handoff</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Copy to Clipboard for AC paste. Better send history UI. Outreach queue page (optional).</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>Content goes to AC manually. Need smooth copy flow.</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>pages/lead-detail.tsx, pages/recommend.tsx</t>
         </is>
       </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I40" s="6" t="inlineStr">
+      <c r="I41" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J40" s="6" t="inlineStr">
+      <c r="J41" s="6" t="inlineStr">
         <is>
           <t>Outreach queue deferred unless &gt;50/day</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>Discovery completeness score</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>Score each conversation 0-100% on new intelligence gathered. Aggregate per agent.</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>See which callers do real discovery vs going through motions.</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>Service + Frontend</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>lib/analysisPipeline.ts, pages/call-inbox.tsx</t>
-        </is>
-      </c>
-      <c r="H41" s="7" t="inlineStr">
-        <is>
-          <t>0.2, 0.11</t>
-        </is>
-      </c>
-      <c r="I41" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J41" s="7" t="inlineStr">
-        <is>
-          <t>Post-core</t>
         </is>
       </c>
     </row>
@@ -2570,37 +2568,37 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Belief journey analytics</t>
+          <t>Discovery completeness score</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Dashboard: hardest beliefs, avg conversations per belief, distribution by cluster.</t>
+          <t>Score each conversation 0-100% on new intelligence gathered. Aggregate per agent.</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>Identify systematic weaknesses in scripts or content.</t>
+          <t>See which callers do real discovery vs going through motions.</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>Frontend + Route</t>
+          <t>Service + Frontend</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>pages/dashboard.tsx or new analytics page</t>
+          <t>lib/analysisPipeline.ts, pages/call-inbox.tsx</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>0.2, 0.11</t>
         </is>
       </c>
       <c r="I42" s="7" t="inlineStr">
@@ -2622,37 +2620,37 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Content effectiveness tracking</t>
+          <t>Belief journey analytics</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Link doc sends to subsequent belief state changes. Build effectiveness map.</t>
+          <t>Dashboard: hardest beliefs, avg conversations per belief, distribution by cluster.</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>Data-driven content strategy. Rewrite underperforming documents.</t>
+          <t>Identify systematic weaknesses in scripts or content.</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Service + Frontend</t>
+          <t>Frontend + Route</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>lib/analysisPipeline.ts, pages/dashboard.tsx</t>
+          <t>pages/dashboard.tsx or new analytics page</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>0.10, 0.11</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="I43" s="7" t="inlineStr">
@@ -2674,37 +2672,37 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Objection memory</t>
+          <t>Content effectiveness tracking</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Track objections across conversations with resolution status. Show in call prep.</t>
+          <t>Link doc sends to subsequent belief state changes. Build effectiveness map.</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>Callers don't re-raise resolved objections. Surface recurring issues.</t>
+          <t>Data-driven content strategy. Rewrite underperforming documents.</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>Schema + Service</t>
+          <t>Service + Frontend</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>lib/db schema changes, lib/analysisPipeline.ts, pages/call-prep.tsx</t>
+          <t>lib/analysisPipeline.ts, pages/dashboard.tsx</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>0.10, 4.1</t>
+          <t>0.10, 0.11</t>
         </is>
       </c>
       <c r="I44" s="7" t="inlineStr">
@@ -2726,37 +2724,37 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Smart next action engine</t>
+          <t>Objection memory</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Multi-step: conversational goal + content + gate check + escalation trigger.</t>
+          <t>Track objections across conversations with resolution status. Show in call prep.</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>From 'what to send' to 'what to do next and why'.</t>
+          <t>Callers don't re-raise resolved objections. Surface recurring issues.</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Schema + Service</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>routes/leads/index.ts, lib/analysisPipeline.ts</t>
+          <t>lib/db schema changes, lib/analysisPipeline.ts, pages/call-prep.tsx</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>0.9, 4.1</t>
+          <t>0.10, 4.1</t>
         </is>
       </c>
       <c r="I45" s="7" t="inlineStr">
@@ -2778,37 +2776,37 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Pre-call briefing card</t>
+          <t>Smart next action engine</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Claude auto-generates 30-second context briefing per lead. Cached, regenerated after each call.</t>
+          <t>Multi-step: conversational goal + content + gate check + escalation trigger.</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>Perfect context in 30 seconds before every call.</t>
+          <t>From 'what to send' to 'what to do next and why'.</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>Service + Frontend</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>routes/leads/index.ts, pages/call-prep.tsx</t>
+          <t>routes/leads/index.ts, lib/analysisPipeline.ts</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>0.2, 0.11, 4.1</t>
+          <t>0.9, 4.1</t>
         </is>
       </c>
       <c r="I46" s="7" t="inlineStr">
@@ -2830,45 +2828,97 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Pre-call briefing card</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Claude auto-generates 30-second context briefing per lead. Cached, regenerated after each call.</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Perfect context in 30 seconds before every call.</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>Service + Frontend</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>routes/leads/index.ts, pages/call-prep.tsx</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>0.2, 0.11, 4.1</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>Post-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
           <t>S7</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>Belief-based lead scoring</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D48" s="7" t="inlineStr">
         <is>
           <t>Score based on qualification gates, universal/cluster/founding beliefs. Formula-driven.</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
+      <c r="E48" s="7" t="inlineStr">
         <is>
           <t>Prioritise genuinely ready leads over email openers.</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
         <is>
           <t>Service + Frontend</t>
         </is>
       </c>
-      <c r="G47" s="7" t="inlineStr">
+      <c r="G48" s="7" t="inlineStr">
         <is>
           <t>routes/leads/index.ts, pages/leads.tsx, pages/call-queue.tsx</t>
         </is>
       </c>
-      <c r="H47" s="7" t="inlineStr">
+      <c r="H48" s="7" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
-      <c r="I47" s="7" t="inlineStr">
+      <c r="I48" s="7" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J47" s="7" t="inlineStr">
+      <c r="J48" s="7" t="inlineStr">
         <is>
           <t>Post-core</t>
         </is>

</xml_diff>

<commit_message>
Update v6 plan with feedback: contact-lead FK, dedup rules, reconciliation
- Explicit bidirectional FK: contacts.lead_id and leads.contact_id
- Dedup hierarchy: exact email > normalised phone > fuzzy name+company
- User-facing merge/skip/update options for fuzzy matches
- Start-of-day reconciliation for uncalled dispatched contacts
- Aircall Dialer Campaign API confirmed available
- dispatch_date field added to contacts schema

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Operational_Readiness_Tracker.xlsx
+++ b/docs/Operational_Readiness_Tracker.xlsx
@@ -1136,7 +1136,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Create pipedrive_sync_config and pipedrive_persons tables.</t>
+          <t>Create contacts table: name, email, phone, company, source_list, upload_batch, dedup_status, campaign_name, dispatch_status (pool/queued/dispatched/called/qualified/archived), dispatch_date, call_attempts, last_call_outcome, callback_date, outreach_paused_until, cool_off_until, aircall_contact_id, pipedrive_person_id, pipedrive_deal_id, lead_id (FK to leads, nullable), created_at, updated_at. Also add contact_id (FK to contacts) on leads table.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1164,7 +1164,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>v6: App owns data. contact_id &lt;-&gt; lead_id bidirectional FK set when first transcript analysed.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1184,7 +1188,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Create lib/integrations/pipedrive/ package with thin fetch wrapper.</t>
+          <t>Upload CSV/Excel. Column mapping. Normalisation (phone, email, name). Dedup hierarchy: 1) exact email match, 2) normalised phone match, 3) fuzzy name+company. Preview shows: X new, Y exact dupes (skip), Z possible matches (user chooses merge/skip/update). Update option refreshes contact details from newer CSV. Store upload history.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1214,7 +1218,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Env: PIPEDRIVE_API_TOKEN, PIPEDRIVE_COMPANY_DOMAIN</t>
+          <t>v6: Dedup hierarchy defined. User chooses merge/skip/update for fuzzy matches.</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1270,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Field mapping in DB, not code</t>
+          <t>v6: Aircall Dialer Campaign API confirmed available. Can create campaigns and add phone numbers programmatically.</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1292,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>POST /pipedrive/sync, GET /status, POST /webhook, GET /persons, POST /link, POST /queue-outreach</t>
+          <t>Campaigns: name, filter criteria on local pool, daily_quota, assigned Aircall user. Dispatch: query contacts, exclude dispatched/cool-off/no-interest, push to Aircall dialer campaign, mark dispatched with dispatch_date. Start-of-day reconciliation: contacts with dispatch_status=dispatched and dispatch_date=yesterday with no call record reset to queued.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1316,7 +1320,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>v6: Includes start-of-day reconciliation for uncalled contacts.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">

</xml_diff>